<commit_message>
Remove H2SO4 and NH4OH
</commit_message>
<xml_diff>
--- a/data/byproduct_markets.xlsx
+++ b/data/byproduct_markets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carolineadkins/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756066AD-19EE-5942-B1F0-931516E42C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F46E8C-D651-9F4F-A022-E5B6649502A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="-26840" windowWidth="27140" windowHeight="21000" xr2:uid="{5BBCCC59-929F-694D-8D6F-26DDD7DC451D}"/>
+    <workbookView xWindow="15500" yWindow="-26600" windowWidth="27140" windowHeight="21000" xr2:uid="{5BBCCC59-929F-694D-8D6F-26DDD7DC451D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="163">
   <si>
     <t>end_use</t>
   </si>
@@ -128,9 +128,6 @@
     <t>Industrial Water Treatment</t>
   </si>
   <si>
-    <t>Pesticide Manufacturing</t>
-  </si>
-  <si>
     <t>CaCO3</t>
   </si>
   <si>
@@ -323,81 +320,12 @@
     <t>Semiconductor Manufacturing</t>
   </si>
   <si>
-    <t>H2SO4</t>
-  </si>
-  <si>
-    <t>Metal Ore Leaching</t>
-  </si>
-  <si>
-    <t>Copper ores</t>
-  </si>
-  <si>
-    <t>Uranium and vanadium ores</t>
-  </si>
-  <si>
-    <t>Other ores</t>
-  </si>
-  <si>
-    <t>Pulp mills and paper products</t>
-  </si>
-  <si>
-    <t>Inorganic pigments, paints, and allied products; industrial organic chemicals; other chemical products4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other inorganic chemicals </t>
-  </si>
-  <si>
-    <t>Synthetic rubber and other plastic materials and synthetics</t>
-  </si>
-  <si>
     <t>Soaps and detergents</t>
   </si>
   <si>
     <t>Nitrogenous Fertilizer Manufacturing</t>
   </si>
   <si>
-    <t>Nitrogenous fertilizers</t>
-  </si>
-  <si>
-    <t>Phosphatic Fertilizer Manufacturing</t>
-  </si>
-  <si>
-    <t>Phosphatic fertilizers</t>
-  </si>
-  <si>
-    <t>Pesticides</t>
-  </si>
-  <si>
-    <t>Other agricultural chemicals</t>
-  </si>
-  <si>
-    <t>Explosives</t>
-  </si>
-  <si>
-    <t>Water-treating compounds</t>
-  </si>
-  <si>
-    <t>Petroleum refining and other petroleum and coal products</t>
-  </si>
-  <si>
-    <t>Rubber and miscellaneous plastic products</t>
-  </si>
-  <si>
-    <t>Nonferrous metals</t>
-  </si>
-  <si>
-    <t>Other primary metals</t>
-  </si>
-  <si>
-    <t>Storage batteries (acid)</t>
-  </si>
-  <si>
-    <t>USGS Minerals Yearbook 2023, Sulfur</t>
-  </si>
-  <si>
-    <t>https://d9-wret.s3.us-west-2.amazonaws.com/assets/palladium/production/s3fs-public/media/files/myb1-2023-sulfu-ERT.xlsx</t>
-  </si>
-  <si>
     <t>K2O</t>
   </si>
   <si>
@@ -570,21 +498,6 @@
   </si>
   <si>
     <t>https://pubs.usgs.gov/periodicals/mcs2026/mcs2026-nitrogen.pdf</t>
-  </si>
-  <si>
-    <t>NH4OH</t>
-  </si>
-  <si>
-    <t>Liquid nitrogen fertilizer</t>
-  </si>
-  <si>
-    <t>Production of household cleaners, organic chemicals, and other miscellaneous uses</t>
-  </si>
-  <si>
-    <t>EPA Water Treatment Chemical Supply Chain Profile, Ammonium Hydroxide</t>
-  </si>
-  <si>
-    <t>https://www.epa.gov/system/files/documents/2023-03/Ammonium%20Hydroxide%20Supply%20Chain%20Profile.pdf</t>
   </si>
   <si>
     <t>P2O5</t>
@@ -1002,7 +915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DF184B4-4209-7340-984B-591345E84F4E}">
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -1015,7 +928,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1041,7 +954,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -1081,7 +994,7 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -1121,7 +1034,7 @@
         <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -1145,7 +1058,7 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -1238,113 +1151,113 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" t="s">
-        <v>42</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" t="s">
         <v>32</v>
-      </c>
-      <c r="G11" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" t="s">
         <v>32</v>
-      </c>
-      <c r="G12" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="F13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" t="s">
         <v>32</v>
-      </c>
-      <c r="G13" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="E14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>32</v>
-      </c>
-      <c r="G14" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" t="s">
         <v>46</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" t="s">
-        <v>47</v>
       </c>
       <c r="E15" s="1">
         <v>1</v>
       </c>
       <c r="F15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" t="s">
         <v>50</v>
-      </c>
-      <c r="G15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" t="s">
         <v>66</v>
-      </c>
-      <c r="B16" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" t="s">
-        <v>67</v>
       </c>
       <c r="D16">
         <v>615</v>
@@ -1354,21 +1267,21 @@
         <v>0.24898785425101214</v>
       </c>
       <c r="F16" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" t="s">
         <v>62</v>
-      </c>
-      <c r="G16" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D17">
         <v>878</v>
@@ -1378,21 +1291,21 @@
         <v>0.3554655870445344</v>
       </c>
       <c r="F17" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" t="s">
         <v>62</v>
-      </c>
-      <c r="G17" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D18">
         <v>446</v>
@@ -1402,21 +1315,21 @@
         <v>0.1805668016194332</v>
       </c>
       <c r="F18" t="s">
+        <v>61</v>
+      </c>
+      <c r="G18" t="s">
         <v>62</v>
-      </c>
-      <c r="G18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19">
         <v>128</v>
@@ -1426,21 +1339,21 @@
         <v>5.1821862348178135E-2</v>
       </c>
       <c r="F19" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" t="s">
         <v>62</v>
-      </c>
-      <c r="G19" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D20">
         <v>47</v>
@@ -1450,21 +1363,21 @@
         <v>1.9028340080971661E-2</v>
       </c>
       <c r="F20" t="s">
+        <v>61</v>
+      </c>
+      <c r="G20" t="s">
         <v>62</v>
-      </c>
-      <c r="G20" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21">
         <v>137</v>
@@ -1474,21 +1387,21 @@
         <v>5.5465587044534415E-2</v>
       </c>
       <c r="F21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" t="s">
         <v>62</v>
-      </c>
-      <c r="G21" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22">
         <v>108</v>
@@ -1498,21 +1411,21 @@
         <v>4.3724696356275301E-2</v>
       </c>
       <c r="F22" t="s">
+        <v>61</v>
+      </c>
+      <c r="G22" t="s">
         <v>62</v>
-      </c>
-      <c r="G22" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23">
         <v>43</v>
@@ -1522,21 +1435,21 @@
         <v>1.7408906882591092E-2</v>
       </c>
       <c r="F23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G23" t="s">
         <v>62</v>
-      </c>
-      <c r="G23" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D24">
         <v>63</v>
@@ -1546,21 +1459,21 @@
         <v>2.5506072874493926E-2</v>
       </c>
       <c r="F24" t="s">
+        <v>61</v>
+      </c>
+      <c r="G24" t="s">
         <v>62</v>
-      </c>
-      <c r="G24" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" t="s">
         <v>69</v>
-      </c>
-      <c r="B25" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" t="s">
-        <v>70</v>
       </c>
       <c r="D25">
         <v>4400</v>
@@ -1570,21 +1483,21 @@
         <v>0.11859838274932614</v>
       </c>
       <c r="F25" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" t="s">
         <v>73</v>
-      </c>
-      <c r="G25" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D26">
         <v>14400</v>
@@ -1594,21 +1507,21 @@
         <v>0.38814016172506738</v>
       </c>
       <c r="F26" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" t="s">
         <v>73</v>
-      </c>
-      <c r="G26" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D27">
         <f>18300</f>
@@ -1619,1592 +1532,1072 @@
         <v>0.49326145552560646</v>
       </c>
       <c r="F27" t="s">
+        <v>72</v>
+      </c>
+      <c r="G27" t="s">
         <v>73</v>
-      </c>
-      <c r="G27" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" t="s">
         <v>76</v>
-      </c>
-      <c r="B28" t="s">
-        <v>83</v>
-      </c>
-      <c r="C28" t="s">
-        <v>77</v>
       </c>
       <c r="E28" s="1">
         <v>0.3</v>
       </c>
       <c r="F28" t="s">
+        <v>79</v>
+      </c>
+      <c r="G28" t="s">
         <v>80</v>
-      </c>
-      <c r="G28" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E29" s="1">
         <v>0.19</v>
       </c>
       <c r="F29" t="s">
+        <v>79</v>
+      </c>
+      <c r="G29" t="s">
         <v>80</v>
-      </c>
-      <c r="G29" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B30" t="s">
         <v>15</v>
       </c>
       <c r="C30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E30" s="1">
         <v>0.19</v>
       </c>
       <c r="F30" t="s">
+        <v>79</v>
+      </c>
+      <c r="G30" t="s">
         <v>80</v>
-      </c>
-      <c r="G30" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E31" s="1">
         <v>0.32</v>
       </c>
       <c r="F31" t="s">
+        <v>79</v>
+      </c>
+      <c r="G31" t="s">
         <v>80</v>
-      </c>
-      <c r="G31" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B32" t="s">
         <v>26</v>
       </c>
       <c r="C32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E32" s="1">
         <v>0.54722222222222228</v>
       </c>
       <c r="F32" t="s">
+        <v>90</v>
+      </c>
+      <c r="G32" t="s">
         <v>91</v>
-      </c>
-      <c r="G32" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B33" t="s">
         <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E33" s="1">
         <v>0.18333333333333332</v>
       </c>
       <c r="F33" t="s">
+        <v>90</v>
+      </c>
+      <c r="G33" t="s">
         <v>91</v>
-      </c>
-      <c r="G33" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E34" s="1">
         <v>0.11388888888888889</v>
       </c>
       <c r="F34" t="s">
+        <v>90</v>
+      </c>
+      <c r="G34" t="s">
         <v>91</v>
-      </c>
-      <c r="G34" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E35" s="1">
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="F35" t="s">
+        <v>90</v>
+      </c>
+      <c r="G35" t="s">
         <v>91</v>
-      </c>
-      <c r="G35" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E36" s="1">
         <v>5.2777777777777778E-2</v>
       </c>
       <c r="F36" t="s">
+        <v>90</v>
+      </c>
+      <c r="G36" t="s">
         <v>91</v>
-      </c>
-      <c r="G36" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E37" s="1">
         <v>4.7222222222222221E-2</v>
       </c>
       <c r="F37" t="s">
+        <v>90</v>
+      </c>
+      <c r="G37" t="s">
         <v>91</v>
-      </c>
-      <c r="G37" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B38" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C38" t="s">
         <v>96</v>
       </c>
-      <c r="D38">
-        <v>275</v>
-      </c>
       <c r="E38" s="1">
-        <f>D38/SUM($D$38:$D$57)</f>
-        <v>4.1704579921140433E-2</v>
+        <v>0.85</v>
       </c>
       <c r="F38" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="G38" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B39" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
         <v>97</v>
       </c>
-      <c r="D39">
-        <v>39</v>
-      </c>
       <c r="E39" s="1">
-        <f t="shared" ref="E39:E57" si="3">D39/SUM($D$38:$D$57)</f>
-        <v>5.9144676979071883E-3</v>
+        <v>0.15</v>
       </c>
       <c r="F39" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="G39" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B40" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="C40" t="s">
-        <v>98</v>
-      </c>
-      <c r="D40">
-        <v>14</v>
+        <v>103</v>
       </c>
       <c r="E40" s="1">
-        <f t="shared" si="3"/>
-        <v>2.1231422505307855E-3</v>
+        <v>0.88</v>
       </c>
       <c r="F40" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G40" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B41" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C41" t="s">
-        <v>99</v>
-      </c>
-      <c r="D41">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E41" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9563239308462238E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F41" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G41" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C42" t="s">
-        <v>100</v>
-      </c>
-      <c r="D42">
-        <v>39</v>
+        <v>105</v>
       </c>
       <c r="E42" s="1">
-        <f t="shared" si="3"/>
-        <v>5.9144676979071883E-3</v>
+        <v>0.02</v>
       </c>
       <c r="F42" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G42" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B43" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C43" t="s">
-        <v>101</v>
-      </c>
-      <c r="D43">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="E43" s="1">
-        <f t="shared" si="3"/>
-        <v>1.016075219896876E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F43" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G43" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="C44" t="s">
-        <v>102</v>
-      </c>
-      <c r="D44">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="E44" s="1">
-        <f t="shared" si="3"/>
-        <v>1.3648771610555051E-3</v>
+        <v>0.01</v>
       </c>
       <c r="F44" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G44" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C45" t="s">
-        <v>103</v>
-      </c>
-      <c r="D45">
-        <v>5</v>
+        <v>108</v>
       </c>
       <c r="E45" s="1">
-        <f t="shared" si="3"/>
-        <v>7.5826508947528053E-4</v>
+        <v>0.01</v>
       </c>
       <c r="F45" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G45" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B46" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="C46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D46">
-        <v>143</v>
+        <v>60</v>
       </c>
       <c r="E46" s="1">
-        <f t="shared" si="3"/>
-        <v>2.1686381558993023E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F46" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="G46" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C47" t="s">
-        <v>107</v>
-      </c>
-      <c r="D47">
-        <v>5430</v>
+        <v>113</v>
       </c>
       <c r="E47" s="1">
-        <f t="shared" si="3"/>
-        <v>0.82347588717015474</v>
+        <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G47" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="B48" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="C48" t="s">
-        <v>108</v>
-      </c>
-      <c r="D48">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="E48" s="1">
-        <f t="shared" si="3"/>
-        <v>1.0615711252653928E-3</v>
+        <v>0.8</v>
       </c>
       <c r="F48" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G48" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C49" t="s">
-        <v>109</v>
-      </c>
-      <c r="D49">
-        <v>20</v>
+        <v>118</v>
       </c>
       <c r="E49" s="1">
-        <f t="shared" si="3"/>
-        <v>3.0330603579011221E-3</v>
+        <v>0.11</v>
       </c>
       <c r="F49" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G49" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C50" t="s">
-        <v>110</v>
-      </c>
-      <c r="D50">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="E50" s="1">
-        <f t="shared" si="3"/>
-        <v>1.2132241431604489E-3</v>
+        <v>0.09</v>
       </c>
       <c r="F50" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G50" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="B51" t="s">
-        <v>40</v>
+        <v>123</v>
       </c>
       <c r="C51" t="s">
-        <v>111</v>
-      </c>
-      <c r="D51">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="E51" s="1">
-        <f t="shared" si="3"/>
-        <v>4.8528965726417957E-3</v>
+        <v>0.48</v>
       </c>
       <c r="F51" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G51" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>112</v>
-      </c>
-      <c r="D52">
-        <v>334</v>
+        <v>118</v>
       </c>
       <c r="E52" s="1">
-        <f t="shared" si="3"/>
-        <v>5.0652107976948739E-2</v>
+        <v>0.22</v>
       </c>
       <c r="F52" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G52" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="B53" t="s">
-        <v>11</v>
+        <v>57</v>
       </c>
       <c r="C53" t="s">
-        <v>113</v>
-      </c>
-      <c r="D53">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="E53" s="1">
-        <f t="shared" si="3"/>
-        <v>6.0661207158022447E-4</v>
+        <v>0.12</v>
       </c>
       <c r="F53" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G53" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="B54" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="C54" t="s">
-        <v>78</v>
-      </c>
-      <c r="D54">
-        <v>11</v>
+        <v>122</v>
       </c>
       <c r="E54" s="1">
-        <f t="shared" si="3"/>
-        <v>1.6681831968456172E-3</v>
+        <v>0.1</v>
       </c>
       <c r="F54" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G54" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="B55" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C55" t="s">
+        <v>60</v>
+      </c>
+      <c r="E55" s="1">
+        <v>0.08</v>
+      </c>
+      <c r="F55" t="s">
         <v>114</v>
       </c>
-      <c r="D55">
-        <v>7</v>
-      </c>
-      <c r="E55" s="1">
-        <f t="shared" si="3"/>
-        <v>1.0615711252653928E-3</v>
-      </c>
-      <c r="F55" t="s">
-        <v>117</v>
-      </c>
       <c r="G55" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="B56" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
-        <v>115</v>
-      </c>
-      <c r="D56">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="E56" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5165301789505612E-4</v>
+        <v>0.42</v>
       </c>
       <c r="F56" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="G56" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="B57" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
       <c r="C57" t="s">
-        <v>116</v>
-      </c>
-      <c r="D57">
-        <v>20</v>
+        <v>126</v>
       </c>
       <c r="E57" s="1">
-        <f t="shared" si="3"/>
-        <v>3.0330603579011221E-3</v>
+        <v>0.37</v>
       </c>
       <c r="F57" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="G57" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B58" t="s">
-        <v>124</v>
+        <v>60</v>
       </c>
       <c r="C58" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="E58" s="1">
-        <v>0.85</v>
+        <v>0.21</v>
       </c>
       <c r="F58" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G58" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>138</v>
       </c>
       <c r="C59" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="E59" s="1">
-        <v>0.15</v>
+        <v>0.45</v>
       </c>
       <c r="F59" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="G59" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B60" t="s">
-        <v>135</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E60" s="1">
-        <v>0.88</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="F60" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G60" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C61" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E61" s="1">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="F61" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G61" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C62" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E62" s="1">
-        <v>0.02</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F62" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G62" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="C63" t="s">
-        <v>130</v>
+        <v>93</v>
       </c>
       <c r="E63" s="1">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="F63" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G63" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B64" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="C64" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E64" s="1">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="F64" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G64" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B65" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C65" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="E65" s="1">
         <v>0.01</v>
       </c>
       <c r="F65" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G65" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B66" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C66" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="E66" s="1">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="F66" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G66" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B67" t="s">
+        <v>39</v>
+      </c>
+      <c r="C67" t="s">
         <v>140</v>
       </c>
-      <c r="C67" t="s">
-        <v>137</v>
-      </c>
       <c r="E67" s="1">
-        <v>1</v>
+        <v>0.23</v>
       </c>
       <c r="F67" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G67" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
+        <v>139</v>
+      </c>
+      <c r="B68" t="s">
+        <v>57</v>
+      </c>
+      <c r="C68" t="s">
         <v>141</v>
       </c>
-      <c r="B68" t="s">
-        <v>59</v>
-      </c>
-      <c r="C68" t="s">
-        <v>23</v>
-      </c>
       <c r="E68" s="1">
-        <v>0.8</v>
+        <v>0.22</v>
       </c>
       <c r="F68" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G68" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B69" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C69" t="s">
         <v>142</v>
       </c>
       <c r="E69" s="1">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
       <c r="F69" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G69" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B70" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C70" t="s">
-        <v>61</v>
+        <v>143</v>
       </c>
       <c r="E70" s="1">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="F70" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G70" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B71" t="s">
-        <v>147</v>
+        <v>59</v>
       </c>
       <c r="C71" t="s">
+        <v>23</v>
+      </c>
+      <c r="E71" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F71" t="s">
         <v>144</v>
       </c>
-      <c r="E71" s="1">
-        <v>0.48</v>
-      </c>
-      <c r="F71" t="s">
-        <v>138</v>
-      </c>
       <c r="G71" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>149</v>
       </c>
       <c r="C72" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E72" s="1">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="F72" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="G72" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B73" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C73" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E73" s="1">
-        <v>0.12</v>
+        <f>0.88-E72</f>
+        <v>0.67</v>
       </c>
       <c r="F73" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="G73" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B74" t="s">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C74" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E74" s="1">
-        <v>0.1</v>
+        <f>1-E72-E73</f>
+        <v>0.12</v>
       </c>
       <c r="F74" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="G74" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="B75" t="s">
-        <v>61</v>
+        <v>154</v>
       </c>
       <c r="C75" t="s">
-        <v>61</v>
+        <v>155</v>
       </c>
       <c r="E75" s="1">
-        <v>0.08</v>
+        <v>0.95</v>
       </c>
       <c r="F75" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="G75" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B76" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C76" t="s">
-        <v>149</v>
+        <v>60</v>
       </c>
       <c r="E76" s="1">
-        <v>0.42</v>
+        <v>0.05</v>
       </c>
       <c r="F76" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G76" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B77" t="s">
-        <v>140</v>
+        <v>64</v>
       </c>
       <c r="C77" t="s">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="E77" s="1">
-        <v>0.37</v>
+        <v>0.65</v>
       </c>
       <c r="F77" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="G77" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B78" t="s">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="C78" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E78" s="1">
-        <v>0.21</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="F78" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="G78" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B79" t="s">
+        <v>11</v>
+      </c>
+      <c r="C79" t="s">
+        <v>160</v>
+      </c>
+      <c r="E79" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="F79" t="s">
+        <v>161</v>
+      </c>
+      <c r="G79" t="s">
         <v>162</v>
-      </c>
-      <c r="C79" t="s">
-        <v>155</v>
-      </c>
-      <c r="E79" s="1">
-        <v>0.45</v>
-      </c>
-      <c r="F79" t="s">
-        <v>160</v>
-      </c>
-      <c r="G79" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C80" t="s">
-        <v>156</v>
+        <v>60</v>
       </c>
       <c r="E80" s="1">
-        <v>0.28000000000000003</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F80" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G80" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>154</v>
-      </c>
-      <c r="B81" t="s">
-        <v>61</v>
-      </c>
-      <c r="C81" t="s">
-        <v>157</v>
-      </c>
-      <c r="E81" s="1">
-        <v>0.09</v>
-      </c>
-      <c r="F81" t="s">
-        <v>160</v>
-      </c>
-      <c r="G81" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>154</v>
-      </c>
-      <c r="B82" t="s">
-        <v>61</v>
-      </c>
-      <c r="C82" t="s">
-        <v>158</v>
-      </c>
-      <c r="E82" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F82" t="s">
-        <v>160</v>
-      </c>
-      <c r="G82" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>154</v>
-      </c>
-      <c r="B83" t="s">
-        <v>40</v>
-      </c>
-      <c r="C83" t="s">
-        <v>103</v>
-      </c>
-      <c r="E83" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="F83" t="s">
-        <v>160</v>
-      </c>
-      <c r="G83" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>154</v>
-      </c>
-      <c r="B84" t="s">
-        <v>37</v>
-      </c>
-      <c r="C84" t="s">
-        <v>159</v>
-      </c>
-      <c r="E84" s="1">
-        <v>0.04</v>
-      </c>
-      <c r="F84" t="s">
-        <v>160</v>
-      </c>
-      <c r="G84" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>154</v>
-      </c>
-      <c r="B85" t="s">
-        <v>58</v>
-      </c>
-      <c r="C85" t="s">
-        <v>145</v>
-      </c>
-      <c r="E85" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="F85" t="s">
-        <v>160</v>
-      </c>
-      <c r="G85" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>154</v>
-      </c>
-      <c r="B86" t="s">
-        <v>60</v>
-      </c>
-      <c r="C86" t="s">
-        <v>23</v>
-      </c>
-      <c r="E86" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="F86" t="s">
-        <v>160</v>
-      </c>
-      <c r="G86" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>163</v>
-      </c>
-      <c r="B87" t="s">
-        <v>40</v>
-      </c>
-      <c r="C87" t="s">
-        <v>164</v>
-      </c>
-      <c r="E87" s="1">
-        <v>0.23</v>
-      </c>
-      <c r="F87" t="s">
-        <v>168</v>
-      </c>
-      <c r="G87" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>163</v>
-      </c>
-      <c r="B88" t="s">
-        <v>58</v>
-      </c>
-      <c r="C88" t="s">
-        <v>165</v>
-      </c>
-      <c r="E88" s="1">
-        <v>0.22</v>
-      </c>
-      <c r="F88" t="s">
-        <v>168</v>
-      </c>
-      <c r="G88" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>163</v>
-      </c>
-      <c r="B89" t="s">
-        <v>40</v>
-      </c>
-      <c r="C89" t="s">
-        <v>166</v>
-      </c>
-      <c r="E89" s="1">
-        <v>0.22</v>
-      </c>
-      <c r="F89" t="s">
-        <v>168</v>
-      </c>
-      <c r="G89" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>163</v>
-      </c>
-      <c r="B90" t="s">
-        <v>61</v>
-      </c>
-      <c r="C90" t="s">
-        <v>167</v>
-      </c>
-      <c r="E90" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="F90" t="s">
-        <v>168</v>
-      </c>
-      <c r="G90" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>163</v>
-      </c>
-      <c r="B91" t="s">
-        <v>60</v>
-      </c>
-      <c r="C91" t="s">
-        <v>23</v>
-      </c>
-      <c r="E91" s="1">
-        <v>0.03</v>
-      </c>
-      <c r="F91" t="s">
-        <v>168</v>
-      </c>
-      <c r="G91" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>170</v>
-      </c>
-      <c r="B92" t="s">
-        <v>173</v>
-      </c>
-      <c r="C92" t="s">
-        <v>171</v>
-      </c>
-      <c r="E92" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="F92" t="s">
-        <v>175</v>
-      </c>
-      <c r="G92" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>170</v>
-      </c>
-      <c r="B93" t="s">
-        <v>104</v>
-      </c>
-      <c r="C93" t="s">
-        <v>172</v>
-      </c>
-      <c r="E93" s="1">
-        <f>0.88-E92</f>
-        <v>0.67</v>
-      </c>
-      <c r="F93" t="s">
-        <v>175</v>
-      </c>
-      <c r="G93" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>170</v>
-      </c>
-      <c r="B94" t="s">
-        <v>40</v>
-      </c>
-      <c r="C94" t="s">
-        <v>174</v>
-      </c>
-      <c r="E94" s="1">
-        <f>1-E92-E93</f>
-        <v>0.12</v>
-      </c>
-      <c r="F94" t="s">
-        <v>175</v>
-      </c>
-      <c r="G94" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>177</v>
-      </c>
-      <c r="B95" t="s">
-        <v>173</v>
-      </c>
-      <c r="C95" t="s">
-        <v>178</v>
-      </c>
-      <c r="E95" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F95" t="s">
-        <v>180</v>
-      </c>
-      <c r="G95" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>177</v>
-      </c>
-      <c r="B96" t="s">
-        <v>61</v>
-      </c>
-      <c r="C96" t="s">
-        <v>179</v>
-      </c>
-      <c r="E96" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F96" t="s">
-        <v>180</v>
-      </c>
-      <c r="G96" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>182</v>
-      </c>
-      <c r="B97" t="s">
-        <v>183</v>
-      </c>
-      <c r="C97" t="s">
-        <v>184</v>
-      </c>
-      <c r="E97" s="1">
-        <v>0.95</v>
-      </c>
-      <c r="F97" t="s">
-        <v>185</v>
-      </c>
-      <c r="G97" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>182</v>
-      </c>
-      <c r="B98" t="s">
-        <v>61</v>
-      </c>
-      <c r="C98" t="s">
-        <v>61</v>
-      </c>
-      <c r="E98" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="F98" t="s">
-        <v>185</v>
-      </c>
-      <c r="G98" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>187</v>
-      </c>
-      <c r="B99" t="s">
-        <v>65</v>
-      </c>
-      <c r="C99" t="s">
-        <v>20</v>
-      </c>
-      <c r="E99" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="F99" t="s">
-        <v>190</v>
-      </c>
-      <c r="G99" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
-        <v>187</v>
-      </c>
-      <c r="B100" t="s">
-        <v>11</v>
-      </c>
-      <c r="C100" t="s">
-        <v>188</v>
-      </c>
-      <c r="E100" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="F100" t="s">
-        <v>190</v>
-      </c>
-      <c r="G100" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>187</v>
-      </c>
-      <c r="B101" t="s">
-        <v>11</v>
-      </c>
-      <c r="C101" t="s">
-        <v>189</v>
-      </c>
-      <c r="E101" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="F101" t="s">
-        <v>190</v>
-      </c>
-      <c r="G101" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>187</v>
-      </c>
-      <c r="B102" t="s">
-        <v>61</v>
-      </c>
-      <c r="C102" t="s">
-        <v>61</v>
-      </c>
-      <c r="E102" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F102" t="s">
-        <v>190</v>
-      </c>
-      <c r="G102" t="s">
-        <v>191</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>